<commit_message>
Added Product Backlog and Sprint Backlog
Added the Product Backlog and Sprint Backlog from planning meeting.
</commit_message>
<xml_diff>
--- a/sprints/Product Backlog.xlsx
+++ b/sprints/Product Backlog.xlsx
@@ -1,51 +1,191 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22325"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonathan Corley\git\SE2-project-repos-sample\sprints\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EC7C4E-5288-43E2-BCCD-AFE8A3B4E981}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0968CCCD-DADA-411A-B4EF-152D35218E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39780" yWindow="1380" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="50">
   <si>
     <t>Priority</t>
   </si>
   <si>
-    <t>Who</t>
-  </si>
-  <si>
-    <t>What</t>
-  </si>
-  <si>
-    <t>Why</t>
-  </si>
-  <si>
     <t>As a…</t>
   </si>
   <si>
-    <t>I want…</t>
+    <t>I want to…</t>
   </si>
   <si>
     <t>So that…</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Create an account</t>
+  </si>
+  <si>
+    <t>I can use the application</t>
+  </si>
+  <si>
+    <t>Log into my account</t>
+  </si>
+  <si>
+    <t>So that I can use my personal data.</t>
+  </si>
+  <si>
+    <t>Create a food item</t>
+  </si>
+  <si>
+    <t>Create a meal item</t>
+  </si>
+  <si>
+    <t>Edit a food item</t>
+  </si>
+  <si>
+    <t>So that I can correct errors.</t>
+  </si>
+  <si>
+    <t>So that I can see available foods to eat.</t>
+  </si>
+  <si>
+    <t>So that I can see available meals to eat.</t>
+  </si>
+  <si>
+    <t>Edit a meal item</t>
+  </si>
+  <si>
+    <t>Search for a specific food item</t>
+  </si>
+  <si>
+    <t>So that I can find foods that I want to eat.</t>
+  </si>
+  <si>
+    <t>Tag food items</t>
+  </si>
+  <si>
+    <t>So that I can group food items by nutrition values.</t>
+  </si>
+  <si>
+    <t>Search for a specific meal item</t>
+  </si>
+  <si>
+    <t>So that I can find a specific meal I want to eat.</t>
+  </si>
+  <si>
+    <t>Tag a meal item</t>
+  </si>
+  <si>
+    <t>So that I can group meal items by nutritional values</t>
+  </si>
+  <si>
+    <t>Create diet plan</t>
+  </si>
+  <si>
+    <t>So that I know what my goals are.</t>
+  </si>
+  <si>
+    <t>Edit a diet plan</t>
+  </si>
+  <si>
+    <t>So that I can change my target goals</t>
+  </si>
+  <si>
+    <t>Select a food item that I've eaten today</t>
+  </si>
+  <si>
+    <t>So I can track what food items I've eaten today.</t>
+  </si>
+  <si>
+    <t>Add a food item to a previous day</t>
+  </si>
+  <si>
+    <t>So I can add food items that I missed that day.</t>
+  </si>
+  <si>
+    <t>Select a meal item that I've eaten today</t>
+  </si>
+  <si>
+    <t>So I can track what meal items I've eaten today.</t>
+  </si>
+  <si>
+    <t>Add a meal item to a previous day</t>
+  </si>
+  <si>
+    <t>So I can add meal items that I missed that day.</t>
+  </si>
+  <si>
+    <t>See what I've eaten by day</t>
+  </si>
+  <si>
+    <t>So that I can know what I've ate.</t>
+  </si>
+  <si>
+    <t>See how many Calories/Nutrition values I have left based on my diet.</t>
+  </si>
+  <si>
+    <t>So that I know what I can choose what I can still eat today.</t>
+  </si>
+  <si>
+    <t>Be informed if I am trying to eat something that will violate my diet plan.</t>
+  </si>
+  <si>
+    <t>So that I can avoid violating my diet plan.</t>
+  </si>
+  <si>
+    <t>See reports of how well I've stuck with my diet plan Daily/Weekly/Monthly/Yearly</t>
+  </si>
+  <si>
+    <t>So that I can know how well I'm doing on my diet.</t>
+  </si>
+  <si>
+    <t>Get recommendations of foods/meals to eat that follow my diet plan</t>
+  </si>
+  <si>
+    <t>So that I can better stick to my diet.</t>
+  </si>
+  <si>
+    <t>Delete Food Item</t>
+  </si>
+  <si>
+    <t>So that I can remove foods that aren't used</t>
+  </si>
+  <si>
+    <t>Delete Meal Item</t>
+  </si>
+  <si>
+    <t>So that I can remove Meals that aren't used</t>
   </si>
 </sst>
 </file>
@@ -87,9 +227,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -370,12 +516,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="126.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -385,7 +531,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -399,14 +545,325 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>3</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D24">
+    <sortCondition ref="A3:A24"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Design Implementation Meeting Updates
Updated planning notes with more detailed descriptions of the system.
Updated the sprint back log with new task assigments
</commit_message>
<xml_diff>
--- a/sprints/Product Backlog.xlsx
+++ b/sprints/Product Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77B26B3-B75A-4157-A7DE-A5E18E9A8A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9F66DA-3E38-455C-8DAE-DBE000E1A5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -523,14 +523,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.5546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="126.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="126.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -544,7 +544,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -558,7 +558,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -572,7 +572,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -586,7 +586,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -600,7 +600,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -614,7 +614,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -628,7 +628,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -642,7 +642,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -656,7 +656,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -670,7 +670,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -684,7 +684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -698,7 +698,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -712,7 +712,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -726,7 +726,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -740,7 +740,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -754,7 +754,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -768,7 +768,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -782,7 +782,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -796,7 +796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -810,7 +810,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -824,7 +824,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -838,7 +838,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>4</v>
       </c>
@@ -852,7 +852,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>4</v>
       </c>
@@ -866,7 +866,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Added CreateMealItemPage.fxml and Controller
I setup the CreateMealItemPage.fxml to basically mimic the
CreateCompositeFoodPage.fxml without the ablity to select a
QuantityCategory since meals will always be by serving.
I also configured the CreateMealItemPageController to mimic the
CreateCompositeFoodPageController since it will provide basically the
same functionality with some small adjustments.
</commit_message>
<xml_diff>
--- a/sprints/Product Backlog.xlsx
+++ b/sprints/Product Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9F66DA-3E38-455C-8DAE-DBE000E1A5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A786132A-FA20-4383-A80D-0D7A85D12EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="1380" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -152,18 +152,6 @@
     <t>So that I can better stick to my diet.</t>
   </si>
   <si>
-    <t>Delete Food Item</t>
-  </si>
-  <si>
-    <t>So that I can remove foods that aren't used</t>
-  </si>
-  <si>
-    <t>Delete Meal Item</t>
-  </si>
-  <si>
-    <t>So that I can remove Meals that aren't used</t>
-  </si>
-  <si>
     <t>Make food items private vs public</t>
   </si>
   <si>
@@ -192,6 +180,18 @@
   </si>
   <si>
     <t>So that I can filter food items by tags.</t>
+  </si>
+  <si>
+    <t>Delete Food Item that have been selected for a day</t>
+  </si>
+  <si>
+    <t>Delete Meal Item that have been selected for a day</t>
+  </si>
+  <si>
+    <t>So that I can remove foods that I added in error</t>
+  </si>
+  <si>
+    <t>So that I can remove Meals that I added in error</t>
   </si>
 </sst>
 </file>
@@ -622,10 +622,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -636,10 +636,10 @@
         <v>4</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -754,7 +754,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -762,13 +762,13 @@
         <v>4</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -776,10 +776,10 @@
         <v>4</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -818,10 +818,10 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -860,10 +860,10 @@
         <v>4</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D24" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -874,10 +874,10 @@
         <v>4</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>